<commit_message>
feat(responsive-search-ads): add Vinkel + Hypotese doc columns (Editor-safe)
Two Inbound-internal columns appended after Final mobile URL, one per RSA row:
the creative angle and the hypothesis behind that ad. Google Ads Editor matches
import columns by name and ignores unrecognised headers, so these (like the LEN
columns) are dropped cleanly on import and never touch the account. Named so they
cannot collide with a real Editor field.

- sheet_layout.py: Vinkel + Hypotese as last two FIELDS (no LEN column).
- fill-sheet.py: write optional per-ad "vinkel"/"hypotese"; documented in both
  ads.json shapes.
- template.xlsx regenerated.
- SKILL.md: column contract + ads.json examples updated, with the
  Editor-ignores-unknown-columns rationale.

Verified: Vinkel/Hypotese land as the last two columns (AW/AX), filled per RSA
row across the multi-RSA shape, real Danish preserved.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/inbound-cph/skills/responsive-search-ads/template.xlsx
+++ b/plugins/inbound-cph/skills/responsive-search-ads/template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AX2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -486,6 +486,8 @@
     <col width="6" customWidth="1" min="46" max="46"/>
     <col width="18" customWidth="1" min="47" max="47"/>
     <col width="18" customWidth="1" min="48" max="48"/>
+    <col width="18" customWidth="1" min="49" max="49"/>
+    <col width="18" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -729,6 +731,16 @@
           <t>Final mobile URL</t>
         </is>
       </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Vinkel</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Hypotese</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="C2" t="inlineStr">

</xml_diff>